<commit_message>
Update literature review figures and study characteristics outputs
</commit_message>
<xml_diff>
--- a/DQA/DQ_Dimensions_Matrix.xlsx
+++ b/DQA/DQ_Dimensions_Matrix.xlsx
@@ -70,7 +70,8 @@
     <t>Consistency</t>
   </si>
   <si>
-    <t>Accuracy /&amp;#10;Correctness</t>
+    <t xml:space="preserve">Accuracy / Correctness / Validity
+</t>
   </si>
   <si>
     <t>Concordance</t>
@@ -82,19 +83,20 @@
     <t>Uniqueness</t>
   </si>
   <si>
-    <t>Temporal&amp;#10;relationships</t>
-  </si>
-  <si>
-    <t>Element level#10;assessment</t>
-  </si>
-  <si>
-    <t>Cross-database&amp;#10;comparison</t>
-  </si>
-  <si>
-    <t>Rule-based&amp;#10;checks</t>
-  </si>
-  <si>
-    <t>Framework&amp;#10;based</t>
+    <t xml:space="preserve">Temporal Relationships
+</t>
+  </si>
+  <si>
+    <t>Element-level Assessment</t>
+  </si>
+  <si>
+    <t>Cross-database or reference-based comparison</t>
+  </si>
+  <si>
+    <t>Rule-based checks</t>
+  </si>
+  <si>
+    <t>Structured DQA framework/programme</t>
   </si>
   <si>
     <t>Ceratti et al., 2008</t>
@@ -115,7 +117,7 @@
     <t>Germany</t>
   </si>
   <si>
-    <t>Khoo &amp; Hasan, 2018</t>
+    <t>Khoo &amp; Hasan, 2019</t>
   </si>
   <si>
     <t>Australia</t>
@@ -160,7 +162,7 @@
     <t>Gadde et al., 2020</t>
   </si>
   <si>
-    <t>Khan et al., 2017</t>
+    <t>Khan et al., 2018</t>
   </si>
   <si>
     <t>Chughtai et al., 2025</t>
@@ -172,7 +174,7 @@
     <t>Ditscheid et al., 2020</t>
   </si>
   <si>
-    <t>Hartmann et al., 2015</t>
+    <t>Hartmann et al., 2016</t>
   </si>
   <si>
     <t>Winkler et al., 2023</t>
@@ -181,7 +183,7 @@
     <t>Lloyd et al., 2025</t>
   </si>
   <si>
-    <t>Wang et al., 2024</t>
+    <t>Wang et al., 2025</t>
   </si>
   <si>
     <t>Total (19)</t>
@@ -884,7 +886,7 @@
       </c>
       <c r="P2" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="107.25">
       <c r="A3" s="9" t="s">
         <v>11</v>
       </c>
@@ -1121,8 +1123,8 @@
       <c r="L7" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="M7" s="17" t="s">
-        <v>30</v>
+      <c r="M7" s="24" t="s">
+        <v>29</v>
       </c>
       <c r="N7" s="18" t="s">
         <v>30</v>
@@ -1421,11 +1423,11 @@
       <c r="L13" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="M13" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="N13" s="18" t="s">
-        <v>30</v>
+      <c r="M13" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N13" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="O13" s="18" t="s">
         <v>30</v>
@@ -1524,8 +1526,8 @@
       <c r="M15" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="N15" s="23" t="s">
-        <v>29</v>
+      <c r="N15" s="18" t="s">
+        <v>30</v>
       </c>
       <c r="O15" s="18" t="s">
         <v>30</v>

</xml_diff>